<commit_message>
Style fixture workbooks with gray header fill and grid borders.
Apply header background and shared border styling from schema_prep ranges when regenerating raw_header and schema fixture workbooks; data band stays uncolored.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/testdata/raw_header/1-row-duplicate-header/workbook.xlsx
+++ b/excel/testdata/raw_header/1-row-duplicate-header/workbook.xlsx
@@ -34,15 +34,20 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDEDED"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -50,12 +55,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF9E9E9E"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF9E9E9E"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF9E9E9E"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF9E9E9E"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="true" applyBorder="true" applyAlignment="false">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true" applyAlignment="false">
+      <alignment/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -327,15 +352,30 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>